<commit_message>
small bugs resolved in frontend app
</commit_message>
<xml_diff>
--- a/src/assets/TruckSample.xlsx
+++ b/src/assets/TruckSample.xlsx
@@ -11,11 +11,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Equipment Number</t>
   </si>
   <si>
+    <t>Plate No</t>
+  </si>
+  <si>
     <t>Equipment Brand</t>
   </si>
   <si>
@@ -46,7 +49,7 @@
     <t>DH346HD673</t>
   </si>
   <si>
-    <t>Ford</t>
+    <t>Benz</t>
   </si>
   <si>
     <t>Trailer</t>
@@ -65,64 +68,13 @@
   </si>
   <si>
     <t>active</t>
-  </si>
-  <si>
-    <t>DH346HD674</t>
-  </si>
-  <si>
-    <t>Kenworth</t>
-  </si>
-  <si>
-    <t>Tanker</t>
-  </si>
-  <si>
-    <t>Owner</t>
-  </si>
-  <si>
-    <t>3Y1SL65848Z411440</t>
-  </si>
-  <si>
-    <t>DH346HD675</t>
-  </si>
-  <si>
-    <t>Peterbilt</t>
-  </si>
-  <si>
-    <t>Flatbed</t>
-  </si>
-  <si>
-    <t>4Y1SL65848Z411440</t>
-  </si>
-  <si>
-    <t>DH346HD677</t>
-  </si>
-  <si>
-    <t>Dodge</t>
-  </si>
-  <si>
-    <t>Forklift</t>
-  </si>
-  <si>
-    <t>Rough Terrain Forklifts</t>
-  </si>
-  <si>
-    <t>4Y1SL65848Z41143333</t>
-  </si>
-  <si>
-    <t>DH346HD6888</t>
-  </si>
-  <si>
-    <t>Freightliner</t>
-  </si>
-  <si>
-    <t>4Y1SL65848</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -150,6 +102,11 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -171,12 +128,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
@@ -190,24 +150,17 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
@@ -425,291 +378,122 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.38"/>
-    <col customWidth="1" min="2" max="3" width="17.13"/>
-    <col customWidth="1" min="4" max="4" width="32.25"/>
-    <col customWidth="1" min="5" max="5" width="20.88"/>
-    <col customWidth="1" min="6" max="7" width="15.5"/>
-    <col customWidth="1" min="9" max="9" width="27.38"/>
+    <col customWidth="1" min="1" max="2" width="18.38"/>
+    <col customWidth="1" min="3" max="4" width="17.13"/>
+    <col customWidth="1" min="5" max="5" width="32.25"/>
+    <col customWidth="1" min="6" max="6" width="20.88"/>
+    <col customWidth="1" min="7" max="8" width="15.5"/>
+    <col customWidth="1" min="10" max="10" width="27.38"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
-      <c r="Z1" s="5"/>
-      <c r="AA1" s="5"/>
+      <c r="K1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="6"/>
+      <c r="Z1" s="6"/>
+      <c r="AA1" s="6"/>
+      <c r="AB1" s="6"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="7">
+        <v>110.0</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="10">
         <v>2015.0</v>
       </c>
-      <c r="H2" s="8">
+      <c r="I2" s="11">
         <v>40.0</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="5"/>
-      <c r="AA2" s="5"/>
+      <c r="K2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6"/>
+      <c r="Z2" s="6"/>
+      <c r="AA2" s="6"/>
+      <c r="AB2" s="6"/>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="7">
-        <v>2019.0</v>
-      </c>
-      <c r="H3" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
-      <c r="AA3" s="5"/>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="10">
-        <v>2019.0</v>
-      </c>
-      <c r="H4" s="11">
-        <v>40.0</v>
-      </c>
-      <c r="I4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="13">
-        <v>2019.0</v>
-      </c>
-      <c r="H5" s="13">
-        <v>40.0</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5"/>
-      <c r="Z5" s="5"/>
-      <c r="AA5" s="5"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="13">
-        <v>2019.0</v>
-      </c>
-      <c r="H6" s="13">
-        <v>40.0</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
-      <c r="AA6" s="5"/>
-    </row>
+    <row r="3" ht="15.75" customHeight="1"/>
+    <row r="4" ht="15.75" customHeight="1"/>
+    <row r="5" ht="15.75" customHeight="1"/>
+    <row r="6" ht="15.75" customHeight="1"/>
     <row r="7" ht="15.75" customHeight="1"/>
     <row r="8" ht="15.75" customHeight="1"/>
     <row r="9" ht="15.75" customHeight="1"/>
@@ -1700,25 +1484,21 @@
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2">
       <formula1>"Ford,Volvo,Kenworth,Peterbilt,Freightliner,International,Mack,Dodge,Hino,Benz"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2">
       <formula1>"Owner,Operator"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2">
       <formula1>"Truck,Trailer,Forklift"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J2:J6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2">
       <formula1>"active,inactive"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2">
       <formula1>"Local,Highway,Flatbed,Refrigerated,Tanker,Lowboy,Counterbalance Forklifts,Electric 3-Wheel Forklifts,Reach Trucks,Pallet Jacks (Manual &amp; Electric),Telehandlers (Telescopic Forklifts),Rough Terrain Forklifts,Side Loader Forklifts,Yard Spotter with Integrat"&amp;"ed Forklift"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>